<commit_message>
Launch tab: location pages plan (USA + UAE country pages, redirect notes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/devsynth-website-seo-2026-10-12.xlsx
+++ b/devsynth-website-seo-2026-10-12.xlsx
@@ -43095,7 +43095,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Training portals are portals; Larimar Training (UAE) is the proof on that page. Old location page; no location pages on the new site.</t>
+          <t>At launch: training portals are portals; Larimar Training (UAE) is the proof on that page. Later: when the UAE country page /locations/uae/ goes live, change this rule's target to /locations/uae/ (edit the rule, never chain redirects).</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -43127,7 +43127,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>EVDC is the EV charging app. Removes the old US state wording.</t>
+          <t>EVDC is the EV charging app. Not the USA country page: EVDC runs across Europe. Removes the old US state wording.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -43191,7 +43191,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Same service, no country page for Albania.</t>
+          <t>Same service. No country page for Albania (Outsorcy is in Kosovo; a one-client country page would be thin).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -43223,7 +43223,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Closest service (wallets and payments). Ali can pick another page.</t>
+          <t>Closest service (wallets and payments). Not the UAE country page: Proud Profits, the crypto app on the old page, is a USA client.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -43371,7 +43371,7 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Location pages (5): Ali decides between these 301s (recommended) and rebuilding them as country pages later.</t>
+          <t>Location pages (5): 301 on launch day (recommended). New country pages /locations/usa/ and /locations/uae/ come after launch, once Ali approves the drafts (Launch tab, Location pages: plan); then only the UAE training-portal rule changes to /locations/uae/.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Master SEO sheet: founder names marked as name-only (navigational), not search targets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/devsynth-website-seo-2026-10-12.xlsx
+++ b/devsynth-website-seo-2026-10-12.xlsx
@@ -7866,7 +7866,7 @@
       <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>commercial</t>
+          <t>navigational</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Yoast focus</t>
+          <t>Yoast focus (person name only: Yoast needs one per page; not a search target, not tracked)</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
@@ -7935,7 +7935,7 @@
       <c r="N19" s="5" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>commercial</t>
+          <t>navigational</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Yoast focus</t>
+          <t>Yoast focus (person name only: Yoast needs one per page; not a search target, not tracked)</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr"/>

</xml_diff>